<commit_message>
Add AX-cluster consolidation (enrich_post_ax_clusters) to GEZE/CHT/EBM reports
Replaces the DINAS-based enrich_master_sub() with a new AX-side function
that uses Abrechnungsstrecken.xlsx (Zusammengefasst in / Hauptabrechnungsstrecke)
to collapse billing sub-rows onto their master. Set-based master detection
prevents dict(zip()) last-value-wins corruption for auftrs appearing in
multiple AX rows.

Results: GEZE 2159 subs removed (2326 rows remain), CHT 38 subs (662 remain),
EBM 0 subs (singleton clusters only). DQ block 8 added to all 3 report builders.

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/billing_report/ebm_dinas_vergleich.xlsx
+++ b/output/billing_report/ebm_dinas_vergleich.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK9"/>
+  <dimension ref="A1:AK10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -639,195 +639,207 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>AX-Cluster-Konsolidierung (Abrechnungsstrecken)</t>
+        </is>
+      </c>
+      <c r="S9" s="4" t="inlineStr">
+        <is>
+          <t>aktiv: ja  |  381 Cluster  |  0 Sub-Rows entfernt  |  7 POST-Rows nicht in AX-Datei</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Auftrags-Nr</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Master-Nr</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Sub-Nr(n)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Anzahl Subs</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Ist Master</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Rech.-Nr</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Sendungsdatum</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Kunde</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Land</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Empf.PLZ</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>Vers.PLZ</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Gew.band</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>Zone</t>
         </is>
       </c>
-      <c r="O9" s="5" t="inlineStr">
+      <c r="O10" s="5" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="P9" s="5" t="inlineStr">
+      <c r="P10" s="5" t="inlineStr">
         <is>
           <t>Basis Menge</t>
         </is>
       </c>
-      <c r="Q9" s="5" t="inlineStr">
+      <c r="Q10" s="5" t="inlineStr">
         <is>
           <t>Basispreis</t>
         </is>
       </c>
-      <c r="R9" s="5" t="inlineStr">
+      <c r="R10" s="5" t="inlineStr">
         <is>
           <t>Eff. Preis</t>
         </is>
       </c>
-      <c r="S9" s="5" t="inlineStr">
+      <c r="S10" s="5" t="inlineStr">
         <is>
           <t>Tonnage kg</t>
         </is>
       </c>
-      <c r="T9" s="5" t="inlineStr">
+      <c r="T10" s="5" t="inlineStr">
         <is>
           <t>Stellplätze</t>
         </is>
       </c>
-      <c r="U9" s="5" t="inlineStr">
+      <c r="U10" s="5" t="inlineStr">
         <is>
           <t>Lademeter</t>
         </is>
       </c>
-      <c r="V9" s="5" t="inlineStr">
+      <c r="V10" s="5" t="inlineStr">
         <is>
           <t>Volumen</t>
         </is>
       </c>
-      <c r="W9" s="5" t="inlineStr">
+      <c r="W10" s="5" t="inlineStr">
         <is>
           <t>Soll EUR</t>
         </is>
       </c>
-      <c r="X9" s="5" t="inlineStr">
+      <c r="X10" s="5" t="inlineStr">
         <is>
           <t>Fracht EUR</t>
         </is>
       </c>
-      <c r="Y9" s="5" t="inlineStr">
+      <c r="Y10" s="5" t="inlineStr">
         <is>
           <t>Diesel EUR</t>
         </is>
       </c>
-      <c r="Z9" s="5" t="inlineStr">
+      <c r="Z10" s="5" t="inlineStr">
         <is>
           <t>Maut EUR</t>
         </is>
       </c>
-      <c r="AA9" s="5" t="inlineStr">
+      <c r="AA10" s="5" t="inlineStr">
         <is>
           <t>Lademittel</t>
         </is>
       </c>
-      <c r="AB9" s="5" t="inlineStr">
+      <c r="AB10" s="5" t="inlineStr">
         <is>
           <t>Peak EUR</t>
         </is>
       </c>
-      <c r="AC9" s="5" t="inlineStr">
+      <c r="AC10" s="5" t="inlineStr">
         <is>
           <t>Neben EUR</t>
         </is>
       </c>
-      <c r="AD9" s="5" t="inlineStr">
+      <c r="AD10" s="5" t="inlineStr">
         <is>
           <t>EUST Zoll</t>
         </is>
       </c>
-      <c r="AE9" s="5" t="inlineStr">
+      <c r="AE10" s="5" t="inlineStr">
         <is>
           <t>Versich.</t>
         </is>
       </c>
-      <c r="AF9" s="5" t="inlineStr">
+      <c r="AF10" s="5" t="inlineStr">
         <is>
           <t>Erlöse</t>
         </is>
       </c>
-      <c r="AG9" s="5" t="inlineStr">
+      <c r="AG10" s="5" t="inlineStr">
         <is>
           <t>Abw. Grund</t>
         </is>
       </c>
-      <c r="AH9" s="5" t="inlineStr">
+      <c r="AH10" s="5" t="inlineStr">
         <is>
           <t>Komplettpreis</t>
         </is>
       </c>
-      <c r="AI9" s="5" t="inlineStr">
+      <c r="AI10" s="5" t="inlineStr">
         <is>
           <t>BI-Split</t>
         </is>
       </c>
-      <c r="AJ9" s="5" t="inlineStr">
+      <c r="AJ10" s="5" t="inlineStr">
         <is>
           <t>DINAS vs BI %</t>
         </is>
       </c>
-      <c r="AK9" s="5" t="inlineStr">
+      <c r="AK10" s="5" t="inlineStr">
         <is>
           <t>DINAS Multi-Row</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="16">
     <mergeCell ref="A3:R3"/>
     <mergeCell ref="S7:AK7"/>
     <mergeCell ref="S5:AK5"/>
@@ -835,9 +847,11 @@
     <mergeCell ref="S6:AK6"/>
     <mergeCell ref="A2:R2"/>
     <mergeCell ref="S4:AK4"/>
+    <mergeCell ref="S9:AK9"/>
     <mergeCell ref="S3:AK3"/>
     <mergeCell ref="S8:AK8"/>
     <mergeCell ref="A5:R5"/>
+    <mergeCell ref="A9:R9"/>
     <mergeCell ref="A1:AK1"/>
     <mergeCell ref="A8:R8"/>
     <mergeCell ref="A6:R6"/>

</xml_diff>